<commit_message>
Docs: back-end package plan in the plan PDF, Gantt file and workbook
- The project management plan PDF gets a package-plan page: a Gantt chart by
  package, start and end dates, what each package waits for, the critical path
  and room to slip. It is now 11 pages and uses the Cloud Cobalt brand and the
  W icon, so it matches the front end and the board.
- Wayfare-Schedule.gan gets the package plan as a second group of tasks, with
  finish-to-start links between cards.
- Wayfare-Planning.xlsx gets Package plan and Package cards sheets.
- The proposal PDF is rebuilt in the same brand. Its text is unchanged.
- The backend board source matches the published board: package ownership
  lock, computed schedule, Gantt chart and critical path.

The dates are a snapshot of 16 Oct 2026 at 2 hours a day for each member. The
board recalculates them. Trello keeps the deadlines.
</commit_message>
<xml_diff>
--- a/docs/Wayfare-Planning.xlsx
+++ b/docs/Wayfare-Planning.xlsx
@@ -10,11 +10,14 @@
     <sheet name="Sprint backlog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sprints" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Milestones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Risk register" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Team" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Package plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Package cards" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Risk register" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Team" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sprint backlog'!$A$4:$J$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Package cards'!$A$4:$M$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +30,7 @@
     <numFmt numFmtId="165" formatCode="d mmm yyyy"/>
     <numFmt numFmtId="166" formatCode="ddd d mmm yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +75,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0014171A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
@@ -111,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,17 +160,22 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -169,6 +183,21 @@
           <bgColor rgb="00E2F3EA"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FBE4E0"/>
+          <bgColor rgb="00FBE4E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00A12C1E"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -4291,6 +4320,2770 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Wayfare: back-end package plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Snapshot of 16 Oct 2026: card sizes S 2, M 4, L 8 hours, 2 hours a day for each member, every calendar day counts. A package starts when the cards it needs are finished. Start and End come from the Backend Board; Cards, Work, Days and Spare are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Cards</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Work (h)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Needs first</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Room (days)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Critical path</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Trello deadline</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Spare (days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Foundation and sign in</t>
+        </is>
+      </c>
+      <c r="C5" s="7">
+        <f>COUNTIF('Package cards'!$A$5:$A$42,A5)</f>
+        <v/>
+      </c>
+      <c r="D5" s="7">
+        <f>SUMIF('Package cards'!$A$5:$A$42,A5,'Package cards'!$E$5:$E$42)</f>
+        <v/>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G5" s="7">
+        <f>F5-E5+1</f>
+        <v/>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>46317</v>
+      </c>
+      <c r="L5" s="7">
+        <f>IF(K5="","",K5-F5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Accounts and profiles</t>
+        </is>
+      </c>
+      <c r="C6" s="7">
+        <f>COUNTIF('Package cards'!$A$5:$A$42,A6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="7">
+        <f>SUMIF('Package cards'!$A$5:$A$42,A6,'Package cards'!$E$5:$E$42)</f>
+        <v/>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>46324</v>
+      </c>
+      <c r="G6" s="7">
+        <f>F6-E6+1</f>
+        <v/>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>A (ready 23 Oct)</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>46353</v>
+      </c>
+      <c r="L6" s="7">
+        <f>IF(K6="","",K6-F6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Browse cars and request one</t>
+        </is>
+      </c>
+      <c r="C7" s="7">
+        <f>COUNTIF('Package cards'!$A$5:$A$42,A7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="7">
+        <f>SUMIF('Package cards'!$A$5:$A$42,A7,'Package cards'!$E$5:$E$42)</f>
+        <v/>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>46326</v>
+      </c>
+      <c r="G7" s="7">
+        <f>F7-E7+1</f>
+        <v/>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>A (ready 23 Oct)</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>46328</v>
+      </c>
+      <c r="L7" s="7">
+        <f>IF(K7="","",K7-F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Rental lifecycle</t>
+        </is>
+      </c>
+      <c r="C8" s="7">
+        <f>COUNTIF('Package cards'!$A$5:$A$42,A8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>SUMIF('Package cards'!$A$5:$A$42,A8,'Package cards'!$E$5:$E$42)</f>
+        <v/>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>46330</v>
+      </c>
+      <c r="G8" s="7">
+        <f>F8-E8+1</f>
+        <v/>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>A (ready 23 Oct) and C (ready 17 Oct)</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>46351</v>
+      </c>
+      <c r="L8" s="7">
+        <f>IF(K8="","",K8-F8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Staff fleet</t>
+        </is>
+      </c>
+      <c r="C9" s="7">
+        <f>COUNTIF('Package cards'!$A$5:$A$42,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>SUMIF('Package cards'!$A$5:$A$42,A9,'Package cards'!$E$5:$E$42)</f>
+        <v/>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>46330</v>
+      </c>
+      <c r="G9" s="7">
+        <f>F9-E9+1</f>
+        <v/>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>A (ready 22 Oct) and B (ready 17 Oct)</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>46358</v>
+      </c>
+      <c r="L9" s="7">
+        <f>IF(K9="","",K9-F9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Staff customers, payments and final test</t>
+        </is>
+      </c>
+      <c r="C10" s="7">
+        <f>COUNTIF('Package cards'!$A$5:$A$42,A10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>SUMIF('Package cards'!$A$5:$A$42,A10,'Package cards'!$E$5:$E$42)</f>
+        <v/>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>46334</v>
+      </c>
+      <c r="G10" s="7">
+        <f>F10-E10+1</f>
+        <v/>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>A (ready 23 Oct) and C (ready 17 Oct)</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>46381</v>
+      </c>
+      <c r="L10" s="7">
+        <f>IF(K10="","",K10-F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="12">
+        <f>SUM(C5:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="12">
+        <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="16">
+        <f>MIN(E5:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="16">
+        <f>MAX(F5:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="12">
+        <f>F11-E11+1</f>
+        <v/>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="10" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="10" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Critical path</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Cards</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Foundation and sign in</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>F1 &gt; F2 &gt; F3 &gt; F5 &gt; F6</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Rental lifecycle</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>R2 &gt; R3 &gt; R4 &gt; A1 &gt; A2 &gt; A4 &gt; A3 &gt; A5 &gt; Q5</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>46330</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Staff customers, payments and final test</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>46331</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>46334</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>If a package on this chain slips a day, the whole back end finishes a day later.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A5:L10">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>$J5="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:L10">
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>AND($L5&lt;&gt;"",$L5&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Wayfare: back-end cards in build order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>One row per open back-end card, grouped by package. Days = End - Start + 1. Spare = Trello due date - End (negative means the plan ends after the Trello date).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Needs first</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Room (days)</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Trello due</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Spare (days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Fix enum typos and add the missing fields</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H5" s="7">
+        <f>G5-F5+1</f>
+        <v/>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="M5" s="7">
+        <f>IF(L5="","",L5-G5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Program.cs setup</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>46313</v>
+      </c>
+      <c r="H6" s="7">
+        <f>G6-F6+1</f>
+        <v/>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="M6" s="7">
+        <f>IF(L6="","",L6-G6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Seed roles, admin account and sample cars</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="H7" s="7">
+        <f>G7-F7+1</f>
+        <v/>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>F1 (A)</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="M7" s="7">
+        <f>IF(L7="","",L7-G7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Authentication and authorization with Identity and JWT</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>46316</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H8" s="7">
+        <f>G8-F8+1</f>
+        <v/>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>F2 (A)</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="M8" s="7">
+        <f>IF(L8="","",L8-G8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Login controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H9" s="7">
+        <f>G9-F9+1</f>
+        <v/>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>F5 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="M9" s="7">
+        <f>IF(L9="","",L9-G9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Create the .http file and the login requests</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H10" s="7">
+        <f>G10-F10+1</f>
+        <v/>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A)</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>46317</v>
+      </c>
+      <c r="M10" s="7">
+        <f>IF(L10="","",L10-G10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 3 test with the front end: sign in and cars</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H11" s="7">
+        <f>G11-F11+1</f>
+        <v/>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F7 (B), C1 (C)</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>46317</v>
+      </c>
+      <c r="M11" s="7">
+        <f>IF(L11="","",L11-G11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Image storage service</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H12" s="7">
+        <f>G12-F12+1</f>
+        <v/>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="M12" s="7">
+        <f>IF(L12="","",L12-G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Register controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H13" s="7">
+        <f>G13-F13+1</f>
+        <v/>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>F4 (B), F5 (A), F1 (A)</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="M13" s="7">
+        <f>IF(L13="","",L13-G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>ChangePassword endpoint</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="H14" s="7">
+        <f>G14-F14+1</f>
+        <v/>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>F5 (A)</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="M14" s="7">
+        <f>IF(L14="","",L14-G14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>GetUserProfile controller and UserProfileDto</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H15" s="7">
+        <f>G15-F15+1</f>
+        <v/>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="M15" s="7">
+        <f>IF(L15="","",L15-G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>UpdateProfile and UpdateLicense endpoints</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H16" s="7">
+        <f>G16-F16+1</f>
+        <v/>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F4 (B), F1 (A)</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>46328</v>
+      </c>
+      <c r="M16" s="7">
+        <f>IF(L16="","",L16-G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Admin profile endpoints</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>46324</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>46324</v>
+      </c>
+      <c r="H17" s="7">
+        <f>G17-F17+1</f>
+        <v/>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>46353</v>
+      </c>
+      <c r="M17" s="7">
+        <f>IF(L17="","",L17-G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>RentalRules service: price, overlap and refund</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H18" s="7">
+        <f>G18-F18+1</f>
+        <v/>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="K18" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="M18" s="7">
+        <f>IF(L18="","",L18-G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Branches endpoint</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H19" s="7">
+        <f>G19-F19+1</f>
+        <v/>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>F2 (A)</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K19" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="M19" s="7">
+        <f>IF(L19="","",L19-G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>ListCar controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H20" s="7">
+        <f>G20-F20+1</f>
+        <v/>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>F3 (A), M1 (C), F5 (A)</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>46312</v>
+      </c>
+      <c r="M20" s="7">
+        <f>IF(L20="","",L20-G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Car details endpoint</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="H21" s="7">
+        <f>G21-F21+1</f>
+        <v/>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>C1 (C)</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K21" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M21" s="7">
+        <f>IF(L21="","",L21-G21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>RentalRequest controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>46324</v>
+      </c>
+      <c r="H22" s="7">
+        <f>G22-F22+1</f>
+        <v/>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>M1 (C), F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>46322</v>
+      </c>
+      <c r="M22" s="7">
+        <f>IF(L22="","",L22-G22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 4 test with the front end: requests, cancel and profile</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="H23" s="7">
+        <f>G23-F23+1</f>
+        <v/>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>R1 (C), R2 (D), R3 (D), R4 (D), P1 (B), P2 (B)</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>46328</v>
+      </c>
+      <c r="M23" s="7">
+        <f>IF(L23="","",L23-G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>ListMyRentals controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="H24" s="7">
+        <f>G24-F24+1</f>
+        <v/>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M24" s="7">
+        <f>IF(L24="","",L24-G24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>CancelRental controller</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H25" s="7">
+        <f>G25-F25+1</f>
+        <v/>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), M1 (C)</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>46324</v>
+      </c>
+      <c r="M25" s="7">
+        <f>IF(L25="","",L25-G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>RefuseRental controller (10% fee)</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H26" s="7">
+        <f>G26-F26+1</f>
+        <v/>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), M1 (C)</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="M26" s="7">
+        <f>IF(L26="","",L26-G26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>AdminListAllRentals controller and DTO</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>46324</v>
+      </c>
+      <c r="H27" s="7">
+        <f>G27-F27+1</f>
+        <v/>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>46335</v>
+      </c>
+      <c r="M27" s="7">
+        <f>IF(L27="","",L27-G27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>ApproveRental controller</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H28" s="7">
+        <f>G28-F28+1</f>
+        <v/>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), M1 (C)</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>46341</v>
+      </c>
+      <c r="M28" s="7">
+        <f>IF(L28="","",L28-G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>HandOverKeys controller</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="H29" s="7">
+        <f>G29-F29+1</f>
+        <v/>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>46343</v>
+      </c>
+      <c r="M29" s="7">
+        <f>IF(L29="","",L29-G29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Rental rejection controller</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>46327</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>46327</v>
+      </c>
+      <c r="H30" s="7">
+        <f>G30-F30+1</f>
+        <v/>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), M1 (C)</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>46345</v>
+      </c>
+      <c r="M30" s="7">
+        <f>IF(L30="","",L30-G30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>RecordReturn controller</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>46328</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>46328</v>
+      </c>
+      <c r="H31" s="7">
+        <f>G31-F31+1</f>
+        <v/>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), F1 (A)</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>46351</v>
+      </c>
+      <c r="M31" s="7">
+        <f>IF(L31="","",L31-G31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 6 test with the front end: the staff workflow</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>46330</v>
+      </c>
+      <c r="H32" s="7">
+        <f>G32-F32+1</f>
+        <v/>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>A2 (D), A3 (D), A4 (D), C4 (E)</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>46348</v>
+      </c>
+      <c r="M32" s="7">
+        <f>IF(L32="","",L32-G32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Staff ListCars controller</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H33" s="7">
+        <f>G33-F33+1</f>
+        <v/>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>F5 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="n">
+        <v>46333</v>
+      </c>
+      <c r="M33" s="7">
+        <f>IF(L33="","",L33-G33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>AddCar controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H34" s="7">
+        <f>G34-F34+1</f>
+        <v/>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>F4 (B), F5 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>46347</v>
+      </c>
+      <c r="M34" s="7">
+        <f>IF(L34="","",L34-G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>DeleteCar controller</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H35" s="7">
+        <f>G35-F35+1</f>
+        <v/>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>F5 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K35" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="n">
+        <v>46355</v>
+      </c>
+      <c r="M35" s="7">
+        <f>IF(L35="","",L35-G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>EditCar controller</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>46324</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H36" s="7">
+        <f>G36-F36+1</f>
+        <v/>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>C4 (E)</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K36" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>46351</v>
+      </c>
+      <c r="M36" s="7">
+        <f>IF(L36="","",L36-G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 7 test with the front end: edit, delete, return</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>46330</v>
+      </c>
+      <c r="H37" s="7">
+        <f>G37-F37+1</f>
+        <v/>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>C5 (E), C6 (E), A5 (D), P5 (B)</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="n">
+        <v>46358</v>
+      </c>
+      <c r="M37" s="7">
+        <f>IF(L37="","",L37-G37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>ListCustomers controller and DTO</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="H38" s="7">
+        <f>G38-F38+1</f>
+        <v/>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A)</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K38" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="n">
+        <v>46331</v>
+      </c>
+      <c r="M38" s="7">
+        <f>IF(L38="","",L38-G38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>VerifyLicense endpoint (staff)</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H39" s="7">
+        <f>G39-F39+1</f>
+        <v/>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), F1 (A)</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K39" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="n">
+        <v>46332</v>
+      </c>
+      <c r="M39" s="7">
+        <f>IF(L39="","",L39-G39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>ListPayments controller, DTO and mapper</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H40" s="7">
+        <f>G40-F40+1</f>
+        <v/>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>F6 (A), F3 (A), M1 (C)</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K40" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="n">
+        <v>46337</v>
+      </c>
+      <c r="M40" s="7">
+        <f>IF(L40="","",L40-G40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 5 test with the front end: staff lists</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="H41" s="7">
+        <f>G41-F41+1</f>
+        <v/>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>P3 (F), C3 (E), A1 (D), M2 (F)</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K41" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="n">
+        <v>46338</v>
+      </c>
+      <c r="M41" s="7">
+        <f>IF(L41="","",L41-G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Final test of the whole system and bug fixing</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>46331</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>46334</v>
+      </c>
+      <c r="H42" s="7">
+        <f>G42-F42+1</f>
+        <v/>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Q2 (A), Q3 (C), Q4 (F), Q5 (D), Q6 (E)</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L42" s="6" t="n">
+        <v>46381</v>
+      </c>
+      <c r="M42" s="7">
+        <f>IF(L42="","",L42-G42)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:M42"/>
+  <conditionalFormatting sqref="A5:M42">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>$K5="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M42">
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>AND($M5&lt;&gt;"",$M5&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4376,17 +7169,17 @@
           <t>7 people, exams, other courses</t>
         </is>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="7">
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="15">
         <f>IF(F5&gt;=6,"High",IF(F5&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4412,17 +7205,17 @@
           <t>New features keep arriving</t>
         </is>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="7">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="15">
         <f>IF(F6&gt;=6,"High",IF(F6&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4448,17 +7241,17 @@
           <t>Different field names or formats</t>
         </is>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="7">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="15">
         <f>IF(F7&gt;=6,"High",IF(F7&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4484,17 +7277,17 @@
           <t>Two customers get the same car</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="7">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="15">
         <f>IF(F8&gt;=6,"High",IF(F8&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4520,17 +7313,17 @@
           <t>Late cards push testing out</t>
         </is>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="7">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="15">
         <f>IF(F9&gt;=6,"High",IF(F9&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4556,17 +7349,17 @@
           <t>Messages missed in a big group</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="7">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="15">
         <f>IF(F10&gt;=6,"High",IF(F10&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4592,17 +7385,17 @@
           <t>Bad merge, deleted files</t>
         </is>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="7">
         <f>D11*E11</f>
         <v/>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="15">
         <f>IF(F11&gt;=6,"High",IF(F11&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4628,17 +7421,17 @@
           <t>Passwords and license data</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="19" t="n">
         <v>3</v>
       </c>
       <c r="F12" s="7">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="15">
         <f>IF(F12&gt;=6,"High",IF(F12&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4664,17 +7457,17 @@
           <t>Testing left to the end</t>
         </is>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="19" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="7">
         <f>D13*E13</f>
         <v/>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="15">
         <f>IF(F13&gt;=6,"High",IF(F13&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4700,17 +7493,17 @@
           <t>Different setups</t>
         </is>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="19" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="7">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="15">
         <f>IF(F14&gt;=6,"High",IF(F14&gt;=3,"Medium","Low"))</f>
         <v/>
       </c>
@@ -4722,13 +7515,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G5:G14">
-    <cfRule type="expression" priority="1" dxfId="1">
+    <cfRule type="expression" priority="1" dxfId="3">
       <formula>$G5="High"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="4">
       <formula>$G5="Medium"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="3">
+    <cfRule type="expression" priority="3" dxfId="5">
       <formula>$G5="Low"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4737,7 +7530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>